<commit_message>
add 2024 including some Russian imports results check
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/output_2024_prepared_final_res_no_Norway.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/output_2024_prepared_final_res_no_Norway.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\02_output_data\02_unidirectional_results\01_paper_IAEE\02_prepared_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00674290-8CE2-4135-A4E8-51205BE75C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39E9C94-1655-46E0-9836-3C144E1A8DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw" sheetId="1" r:id="rId1"/>
@@ -1556,15 +1556,6 @@
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="thick">
           <color theme="0"/>
@@ -1604,6 +1595,15 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
@@ -2635,10 +2635,10 @@
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{0E30B145-4D3F-4FAD-BD41-21ABAB04B6EC}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{757D861D-FB27-46FF-B0C9-F12A4872D22A}" name="Flow (GWh)" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{757D861D-FB27-46FF-B0C9-F12A4872D22A}" name="Flow (GWh)" dataDxfId="8">
       <calculatedColumnFormula>VLOOKUP($A2,Raw!$C$3:$E$454,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B42BA0CA-AAF3-4240-B01E-874DB68E1F64}" name="Share" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{B42BA0CA-AAF3-4240-B01E-874DB68E1F64}" name="Share" dataDxfId="7">
       <calculatedColumnFormula>VLOOKUP($A2,Raw!$C$3:$E$454,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2651,10 +2651,10 @@
   <autoFilter ref="A1:C17" xr:uid="{3417075B-B51B-429B-8BA8-43E190BF8519}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{A239A1DC-0210-4956-ABE7-EF6CDA5A30E2}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{322E7DE0-B95E-46AC-9403-C71D0E63B73A}" name="Flow (GWh)" dataDxfId="2">
+    <tableColumn id="2" xr3:uid="{322E7DE0-B95E-46AC-9403-C71D0E63B73A}" name="Flow (GWh)" dataDxfId="6">
       <calculatedColumnFormula>VLOOKUP(LNG_Import_use!$A2,Raw!$C$3:$E$454,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E19B88D8-3893-4610-AB1D-CF00C32B1D5C}" name="Share" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{E19B88D8-3893-4610-AB1D-CF00C32B1D5C}" name="Share" dataDxfId="5">
       <calculatedColumnFormula>VLOOKUP(LNG_Import_use!$A2,Raw!$C$3:$E$429,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2667,7 +2667,7 @@
   <autoFilter ref="A1:B103" xr:uid="{A8372A6F-EB83-42B1-A6B1-D9A865C31E2A}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D3B0A0F4-AE4B-4C05-803A-8265FB2E0BEC}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{3D272239-DFA1-4C23-990B-17340DB0F202}" name="Flow (GWh)" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{3D272239-DFA1-4C23-990B-17340DB0F202}" name="Flow (GWh)" dataDxfId="4">
       <calculatedColumnFormula>SUMIFS(Raw!$D$2:$D$454,Raw!$C$2:$C$454,"*"&amp;LNG_Sources!$A2&amp;"*")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2676,11 +2676,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}" name="Table7" displayName="Table7" ref="D1:E6" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}" name="Table7" displayName="Table7" ref="D1:E6" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2">
   <autoFilter ref="D1:E6" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{4B792274-18C2-4C26-B54A-695915F3118E}" name="Region"/>
-    <tableColumn id="2" xr3:uid="{46C98E86-4B19-4A99-BF1A-17F24AC916F1}" name="Flow (GWh)" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{46C98E86-4B19-4A99-BF1A-17F24AC916F1}" name="Flow (GWh)" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2691,7 +2691,7 @@
   <autoFilter ref="A1:B38" xr:uid="{8121B5DA-0937-487A-A3DF-77ACBB8999F9}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{03B06CF4-5F36-4B7E-8CC9-8D06BB4532D5}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{1AD1E774-B856-4665-89D5-9C7DC08BC3A8}" name="Flow (GWh)" dataDxfId="3">
+    <tableColumn id="2" xr3:uid="{1AD1E774-B856-4665-89D5-9C7DC08BC3A8}" name="Flow (GWh)" dataDxfId="0">
       <calculatedColumnFormula>VLOOKUP($A2,Raw!$C$3:$E$429,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>